<commit_message>
Fix: correct Singlish input type categories to match actual row content
</commit_message>
<xml_diff>
--- a/IT23225060_Assignment 1 - Test cases.xlsx
+++ b/IT23225060_Assignment 1 - Test cases.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Includes question words/markers like "wage?" or "da?"</t>
+          <t>Contains question marker "nadda" and question structure</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Includes question words/markers like "wage?" or "da?"</t>
+          <t>Contains question word "puluwanda?"</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Question Forms</t>
+          <t>Command Forms</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Includes question words/markers like "wage?" or "da?"</t>
+          <t>Uses imperative commands "danna epa", "idanna"</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Uses imperative/command structures like "denna" or "karanna"</t>
+          <t>Uses imperative commands "open karala", "ewanna"</t>
         </is>
       </c>
     </row>
@@ -710,12 +710,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Command Forms</t>
+          <t>Greetings</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Uses imperative/command structures like "denna" or "karanna"</t>
+          <t>Contains greeting phrase "suba udasanak"</t>
         </is>
       </c>
     </row>
@@ -752,12 +752,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Command Forms</t>
+          <t>Greetings</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Uses imperative/command structures like "denna" or "karanna"</t>
+          <t>Contains greeting "ayubowan"</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Greetings</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Contains greeting words like "Subada", "salam"</t>
+          <t>Polite request using "karunakara" and "help denna"</t>
         </is>
       </c>
     </row>
@@ -836,12 +836,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Greetings</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Contains greeting words like "Subada", "salam"</t>
+          <t>Polite request using "feedback ekak denna"</t>
         </is>
       </c>
     </row>
@@ -878,12 +878,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Responses</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Polite requests using "karunakara", "ane", or "poddak"</t>
+          <t>Response word "hari" acknowledging agreement</t>
         </is>
       </c>
     </row>
@@ -920,12 +920,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Responses</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Polite requests using "karunakara", "ane", or "poddak"</t>
+          <t>Response word "ow" acknowledging understanding</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Repeated Words</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Polite requests using "karunakara", "ane", or "poddak"</t>
+          <t>Contains repeated word "poddak poddak"</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Responses</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Response words like "hari", "ow"</t>
+          <t>Contains punctuation "...?" (ellipsis + question mark)</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Responses</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Response words like "hari", "ow"</t>
+          <t>Contains exclamation mark "ane!"</t>
         </is>
       </c>
     </row>
@@ -1088,12 +1088,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Repeated Words</t>
+          <t>Romanization/Spelling Variants</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Contains reduplicated words for emphasis (e.g. "dhuk dhuk")</t>
+          <t>Informal romanized spelling "ratata adarei"</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Repeated Words</t>
+          <t>Romanization/Spelling Variants</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Contains reduplicated words for emphasis (e.g. "dhuk dhuk")</t>
+          <t>Spelling variant with mixed Singlish/English and abbreviation "pls"</t>
         </is>
       </c>
     </row>
@@ -1172,12 +1172,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Isolated English Word Insertions</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Contains punctuation like ..., -, !</t>
+          <t>Embeds isolated English word "class" in Sinhala sentence</t>
         </is>
       </c>
     </row>
@@ -1210,12 +1210,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Isolated English Word Insertions</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Contains punctuation like ..., -, !</t>
+          <t>Embeds isolated English word "book" in Sinhala sentence</t>
         </is>
       </c>
     </row>
@@ -1252,12 +1252,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Multi-Word English Phrases</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Contains punctuation like ..., -, !</t>
+          <t>Contains multi-word English phrase "today afternoon meeting"</t>
         </is>
       </c>
     </row>
@@ -1294,12 +1294,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Romanization/Spelling Variants</t>
+          <t>Multi-Word English Phrases</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
+          <t>Contains multi-word English phrase "send me the link"</t>
         </is>
       </c>
     </row>
@@ -1336,12 +1336,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Romanization/Spelling Variants</t>
+          <t>English Digital Terms</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
+          <t>Contains digital term "link" and "open"</t>
         </is>
       </c>
     </row>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Romanization/Spelling Variants</t>
+          <t>English Digital Terms</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
+          <t>Contains digital term "email"</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Romanization/Spelling Variants</t>
+          <t>Platform/App Names</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
+          <t>Contains platform name "WhatsApp"</t>
         </is>
       </c>
     </row>
@@ -1462,12 +1462,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Isolated English Word Insertions</t>
+          <t>Platform/App Names</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Embeds single English words like "breakfast", "cafe"</t>
+          <t>Contains platform name "Instagram"</t>
         </is>
       </c>
     </row>
@@ -1500,12 +1500,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Isolated English Word Insertions</t>
+          <t>English Abbreviations/Acronyms</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Embeds single English words like "download", "file"</t>
+          <t>Contains acronym "ASAP"</t>
         </is>
       </c>
     </row>
@@ -1542,12 +1542,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Multi-Word English Phrases</t>
+          <t>English Abbreviations/Acronyms</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Embeds English phrases like "feeling so tired"</t>
+          <t>Contains acronym "BTW"</t>
         </is>
       </c>
     </row>
@@ -1584,12 +1584,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Multi-Word English Phrases</t>
+          <t>English Clipped Forms</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Embeds English phrases like "at the corner shop"</t>
+          <t>Contains clipped English word "info" (from information)</t>
         </is>
       </c>
     </row>
@@ -1626,12 +1626,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>English Digital Terms</t>
+          <t>English Clipped Forms</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Contains tech/digital terms like "WiFi signal"</t>
+          <t>Contains clipped English word "photo" (from photograph)</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>English Digital Terms</t>
+          <t>Place Names Embedded</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Contains tech/digital terms like "laptop", "network"</t>
+          <t>Contains place name "Kandy"</t>
         </is>
       </c>
     </row>
@@ -1710,12 +1710,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Platform/App Names</t>
+          <t>Place Names Embedded</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Mentions platforms like "discord"</t>
+          <t>Contains place name "Colombo"</t>
         </is>
       </c>
     </row>
@@ -1752,12 +1752,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Platform/App Names</t>
+          <t>Person Names Embedded</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Mentions platforms like "Messenger", "LinkedIn"</t>
+          <t>Contains person name "Nimal"</t>
         </is>
       </c>
     </row>
@@ -1794,12 +1794,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms</t>
+          <t>Person Names Embedded</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Contains acronyms/abbreviations like "Passport" or "ID"</t>
+          <t>Contains person name "Amali"</t>
         </is>
       </c>
     </row>
@@ -1836,12 +1836,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Contains acronyms/abbreviations like "JSON", "XML", "API"</t>
+          <t>Contains numeric suffix "2nd"</t>
         </is>
       </c>
     </row>
@@ -1878,12 +1878,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>English Clipped Forms</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Contains clipped words like "admin"</t>
+          <t>Contains number "101"</t>
         </is>
       </c>
     </row>
@@ -1920,12 +1920,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>English Clipped Forms</t>
+          <t>Inputs with Currency</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Contains clipped words like "exam", "essay"</t>
+          <t>Contains currency notation "Rs.500"</t>
         </is>
       </c>
     </row>
@@ -1962,12 +1962,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Place Names Embedded</t>
+          <t>Inputs with Currency</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Mentions specific locations like "Thailand"</t>
+          <t>Contains currency notation "USD 20"</t>
         </is>
       </c>
     </row>
@@ -2004,12 +2004,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Place Names Embedded</t>
+          <t>Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Mentions specific locations like "Malaysia", "Kandy"</t>
+          <t>Contains time format "8.15 AM"</t>
         </is>
       </c>
     </row>
@@ -2046,12 +2046,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Person Names Embedded</t>
+          <t>Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Contains names like "Jayasinghe"</t>
+          <t>Contains time format "14:45" (24-hour)</t>
         </is>
       </c>
     </row>
@@ -2088,12 +2088,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Person Names Embedded</t>
+          <t>Inputs with Dates</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Contains names like "Chathura", "Nishantha"</t>
+          <t>Contains date format "2026-06-15" (ISO format)</t>
         </is>
       </c>
     </row>
@@ -2130,12 +2130,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>Inputs with Dates</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Contains numbers like "95n 100yama"</t>
+          <t>Contains date format "15/07/2026" (DD/MM/YYYY)</t>
         </is>
       </c>
     </row>
@@ -2172,12 +2172,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Contains numbers like "5th", "48 hours"</t>
+          <t>Contains measurement unit "3500 meters"</t>
         </is>
       </c>
     </row>
@@ -2214,12 +2214,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
+          <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Contains currency like "Swiss Francs 200"</t>
+          <t>Contains measurement unit "2 liters"</t>
         </is>
       </c>
     </row>
@@ -2252,12 +2252,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
+          <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Contains currency like "INR 5000", "AUD"</t>
+          <t>Contains slang "machan" (buddy) with casual phrasing</t>
         </is>
       </c>
     </row>
@@ -2290,12 +2290,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
+          <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Contains time formats like "8.15AM"</t>
+          <t>Contains casual exclamation "aiyo" with informal tone</t>
         </is>
       </c>
     </row>
@@ -2328,12 +2328,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
+          <t>Inputs with Special Characters</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Contains time formats like "2.30pm", "14:45"</t>
+          <t>Contains special character "@" in "@nimal"</t>
         </is>
       </c>
     </row>
@@ -2366,12 +2366,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
+          <t>Inputs with Special Characters</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Contains date formats like "2026-06-15"</t>
+          <t>Contains special characters in email format "nimal123@gmail.com"</t>
         </is>
       </c>
     </row>
@@ -2404,12 +2404,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
+          <t>Inputs with Emojis</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Contains date formats like "June 30", "15/07/2026"</t>
+          <t>Contains emoji character embedded in Sinhala text</t>
         </is>
       </c>
     </row>
@@ -2442,12 +2442,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
+          <t>Inputs with Emojis</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Contains measurement units like "2 hours", "meters", "kilograms"</t>
+          <t>Contains emoji character embedded in Sinhala text</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2484,12 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
+          <t>Inputs with Code-Switching</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Contains measurement units like "meters", "kilograms", "220V"</t>
+          <t>Full code-switching between Sinhala and English: "then call me asap, otherwise text karanna"</t>
         </is>
       </c>
     </row>
@@ -2526,12 +2526,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
+          <t>Inputs with Code-Switching</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Uses slang/informal language</t>
+          <t>Full code-switching with English phrase: "buddy, and this is urgent pls"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace blank actual outputs with placeholder
</commit_message>
<xml_diff>
--- a/IT23225060_Assignment 1 - Test cases.xlsx
+++ b/IT23225060_Assignment 1 - Test cases.xlsx
@@ -534,10 +534,14 @@
           <t>ඔයා කොහොමද? today class එක යන්නේ නැද්ද, asap reply දෙන්න.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>No output captured</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -547,7 +551,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Contains question marker "nadda" and question structure</t>
+          <t>Includes question words/markers like "wage?" or "da?"</t>
         </is>
       </c>
     </row>
@@ -579,7 +583,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -589,7 +593,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Contains question word "puluwanda?"</t>
+          <t>Includes question words/markers like "wage?" or "da?"</t>
         </is>
       </c>
     </row>
@@ -621,17 +625,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Command Forms</t>
+          <t>Question Forms</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Uses imperative commands "danna epa", "idanna"</t>
+          <t>Includes question words/markers like "wage?" or "da?"</t>
         </is>
       </c>
     </row>
@@ -658,12 +662,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>දොර එක දාන්න එපා, මෙතන ඉදන්න.</t>
+          <t>No output captured</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -673,7 +677,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Uses imperative commands "open karala", "ewanna"</t>
+          <t>Uses imperative/command structures like "denna" or "karanna"</t>
         </is>
       </c>
     </row>
@@ -705,17 +709,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Greetings</t>
+          <t>Command Forms</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Contains greeting phrase "suba udasanak"</t>
+          <t>Uses imperative/command structures like "denna" or "karanna"</t>
         </is>
       </c>
     </row>
@@ -747,17 +751,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Greetings</t>
+          <t>Command Forms</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Contains greeting "ayubowan"</t>
+          <t>Uses imperative/command structures like "denna" or "karanna"</t>
         </is>
       </c>
     </row>
@@ -789,17 +793,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Greetings</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Polite request using "karunakara" and "help denna"</t>
+          <t>Contains greeting words like "Subada", "salam"</t>
         </is>
       </c>
     </row>
@@ -826,22 +830,22 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>කරුණාකර පොඩ්ඩක් හෙල්ප් දෙන්න.</t>
+          <t>මේක බලලා feedback එකක් දෙන්න.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Requests</t>
+          <t>Greetings</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Polite request using "feedback ekak denna"</t>
+          <t>Contains greeting words like "Subada", "salam"</t>
         </is>
       </c>
     </row>
@@ -868,22 +872,22 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>මේක බලලා feedback එකක් දෙන්න.</t>
+          <t>හරි, මම ඒක කරන්නම්.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Responses</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Response word "hari" acknowledging agreement</t>
+          <t>Polite requests using "karunakara", "ane", or "poddak"</t>
         </is>
       </c>
     </row>
@@ -910,22 +914,22 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>හරි, මම ඒක කරන්නම්.</t>
+          <t>No output captured</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Responses</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Response word "ow" acknowledging understanding</t>
+          <t>Polite requests using "karunakara", "ane", or "poddak"</t>
         </is>
       </c>
     </row>
@@ -957,17 +961,17 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Repeated Words</t>
+          <t>Requests</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Contains repeated word "poddak poddak"</t>
+          <t>Polite requests using "karunakara", "ane", or "poddak"</t>
         </is>
       </c>
     </row>
@@ -999,17 +1003,17 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Responses</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Contains punctuation "...?" (ellipsis + question mark)</t>
+          <t>Response words like "hari", "ow"</t>
         </is>
       </c>
     </row>
@@ -1041,17 +1045,17 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Inputs with Punctuation Marks</t>
+          <t>Responses</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Contains exclamation mark "ane!"</t>
+          <t>Response words like "hari", "ow"</t>
         </is>
       </c>
     </row>
@@ -1083,17 +1087,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Romanization/Spelling Variants</t>
+          <t>Repeated Words</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Informal romanized spelling "ratata adarei"</t>
+          <t>Contains reduplicated words for emphasis (e.g. "dhuk dhuk")</t>
         </is>
       </c>
     </row>
@@ -1125,17 +1129,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Romanization/Spelling Variants</t>
+          <t>Repeated Words</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Spelling variant with mixed Singlish/English and abbreviation "pls"</t>
+          <t>Contains reduplicated words for emphasis (e.g. "dhuk dhuk")</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1171,17 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Isolated English Word Insertions</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Embeds isolated English word "class" in Sinhala sentence</t>
+          <t>Contains punctuation like ..., -, !</t>
         </is>
       </c>
     </row>
@@ -1202,20 +1206,24 @@
           <t>මම අද class යන්න ඕන.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>No output captured</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Isolated English Word Insertions</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Embeds isolated English word "book" in Sinhala sentence</t>
+          <t>Contains punctuation like ..., -, !</t>
         </is>
       </c>
     </row>
@@ -1247,17 +1255,17 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Multi-Word English Phrases</t>
+          <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Contains multi-word English phrase "today afternoon meeting"</t>
+          <t>Contains punctuation like ..., -, !</t>
         </is>
       </c>
     </row>
@@ -1289,17 +1297,17 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Multi-Word English Phrases</t>
+          <t>Romanization/Spelling Variants</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Contains multi-word English phrase "send me the link"</t>
+          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
         </is>
       </c>
     </row>
@@ -1331,17 +1339,17 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>English Digital Terms</t>
+          <t>Romanization/Spelling Variants</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Contains digital term "link" and "open"</t>
+          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
         </is>
       </c>
     </row>
@@ -1373,17 +1381,17 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>English Digital Terms</t>
+          <t>Romanization/Spelling Variants</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Contains digital term "email"</t>
+          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
         </is>
       </c>
     </row>
@@ -1415,17 +1423,17 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Platform/App Names</t>
+          <t>Romanization/Spelling Variants</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Contains platform name "WhatsApp"</t>
+          <t>Contains unusual spelling variants (e.g., "adorey", "asay")</t>
         </is>
       </c>
     </row>
@@ -1457,17 +1465,17 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Platform/App Names</t>
+          <t>Isolated English Word Insertions</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Contains platform name "Instagram"</t>
+          <t>Embeds single English words like "breakfast", "cafe"</t>
         </is>
       </c>
     </row>
@@ -1492,20 +1500,24 @@
           <t>ඉන්ස්ටග්‍රෑම් story එක බලන්න.</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Instagram story එක බලන්න.</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms</t>
+          <t>Isolated English Word Insertions</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Contains acronym "ASAP"</t>
+          <t>Embeds single English words like "download", "file"</t>
         </is>
       </c>
     </row>
@@ -1537,17 +1549,17 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms</t>
+          <t>Multi-Word English Phrases</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Contains acronym "BTW"</t>
+          <t>Embeds English phrases like "feeling so tired"</t>
         </is>
       </c>
     </row>
@@ -1579,17 +1591,17 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>English Clipped Forms</t>
+          <t>Multi-Word English Phrases</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Contains clipped English word "info" (from information)</t>
+          <t>Embeds English phrases like "at the corner shop"</t>
         </is>
       </c>
     </row>
@@ -1621,17 +1633,17 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>English Clipped Forms</t>
+          <t>English Digital Terms</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Contains clipped English word "photo" (from photograph)</t>
+          <t>Contains tech/digital terms like "WiFi signal"</t>
         </is>
       </c>
     </row>
@@ -1663,17 +1675,17 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Place Names Embedded</t>
+          <t>English Digital Terms</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Contains place name "Kandy"</t>
+          <t>Contains tech/digital terms like "laptop", "network"</t>
         </is>
       </c>
     </row>
@@ -1705,17 +1717,17 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Place Names Embedded</t>
+          <t>Platform/App Names</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Contains place name "Colombo"</t>
+          <t>Mentions platforms like "discord"</t>
         </is>
       </c>
     </row>
@@ -1747,17 +1759,17 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Person Names Embedded</t>
+          <t>Platform/App Names</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Contains person name "Nimal"</t>
+          <t>Mentions platforms like "Messenger", "LinkedIn"</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1801,17 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Person Names Embedded</t>
+          <t>English Abbreviations/Acronyms</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Contains person name "Amali"</t>
+          <t>Contains acronyms/abbreviations like "Passport" or "ID"</t>
         </is>
       </c>
     </row>
@@ -1831,17 +1843,17 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>English Abbreviations/Acronyms</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Contains numeric suffix "2nd"</t>
+          <t>Contains acronyms/abbreviations like "JSON", "XML", "API"</t>
         </is>
       </c>
     </row>
@@ -1873,17 +1885,17 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
+          <t>English Clipped Forms</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Contains number "101"</t>
+          <t>Contains clipped words like "admin"</t>
         </is>
       </c>
     </row>
@@ -1915,17 +1927,17 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
+          <t>English Clipped Forms</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Contains currency notation "Rs.500"</t>
+          <t>Contains clipped words like "exam", "essay"</t>
         </is>
       </c>
     </row>
@@ -1957,17 +1969,17 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
+          <t>Place Names Embedded</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Contains currency notation "USD 20"</t>
+          <t>Mentions specific locations like "Thailand"</t>
         </is>
       </c>
     </row>
@@ -1994,22 +2006,22 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>USD 20 අපිට ඕනේ.</t>
+          <t>No output captured</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
+          <t>Place Names Embedded</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Contains time format "8.15 AM"</t>
+          <t>Mentions specific locations like "Malaysia", "Kandy"</t>
         </is>
       </c>
     </row>
@@ -2041,17 +2053,17 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
+          <t>Person Names Embedded</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Contains time format "14:45" (24-hour)</t>
+          <t>Contains names like "Jayasinghe"</t>
         </is>
       </c>
     </row>
@@ -2083,17 +2095,17 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
+          <t>Person Names Embedded</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Contains date format "2026-06-15" (ISO format)</t>
+          <t>Contains names like "Chathura", "Nishantha"</t>
         </is>
       </c>
     </row>
@@ -2125,17 +2137,17 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Contains date format "15/07/2026" (DD/MM/YYYY)</t>
+          <t>Contains numbers like "95n 100yama"</t>
         </is>
       </c>
     </row>
@@ -2167,17 +2179,17 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Contains measurement unit "3500 meters"</t>
+          <t>Contains numbers like "5th", "48 hours"</t>
         </is>
       </c>
     </row>
@@ -2209,17 +2221,17 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
+          <t>Inputs with Currency</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Contains measurement unit "2 liters"</t>
+          <t>Contains currency like "Swiss Francs 200"</t>
         </is>
       </c>
     </row>
@@ -2244,20 +2256,24 @@
           <t>bottle එකේ 2 liters තියෙනවා.</t>
         </is>
       </c>
-      <c r="E43" s="2" t="n"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>bottle එකේ 2 ලිටර්ස් තියෙනවා.</t>
+        </is>
+      </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
+          <t>Inputs with Currency</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Contains slang "machan" (buddy) with casual phrasing</t>
+          <t>Contains currency like "INR 5000", "AUD"</t>
         </is>
       </c>
     </row>
@@ -2282,20 +2298,24 @@
           <t>මචං, පොඩ්ඩක් ඉන්න.</t>
         </is>
       </c>
-      <c r="E44" s="2" t="n"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>No output captured</t>
+        </is>
+      </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
+          <t>Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Contains casual exclamation "aiyo" with informal tone</t>
+          <t>Contains time formats like "8.15AM"</t>
         </is>
       </c>
     </row>
@@ -2320,20 +2340,24 @@
           <t>අයියෝ, එහෙම කරන්න එපා, නෙවෙයි කියලා හිතන්න එපා.</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>No output captured</t>
+        </is>
+      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Inputs with Special Characters</t>
+          <t>Inputs with Time Formats</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Contains special character "@" in "@nimal"</t>
+          <t>Contains time formats like "2.30pm", "14:45"</t>
         </is>
       </c>
     </row>
@@ -2358,20 +2382,24 @@
           <t>මට @nimal ට message එකක් දන්න.</t>
         </is>
       </c>
-      <c r="E46" s="2" t="n"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>මට @නිමල් ට message එකක් දාන්න.</t>
+        </is>
+      </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Inputs with Special Characters</t>
+          <t>Inputs with Dates</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Contains special characters in email format "nimal123@gmail.com"</t>
+          <t>Contains date formats like "2026-06-15"</t>
         </is>
       </c>
     </row>
@@ -2396,20 +2424,24 @@
           <t>email id එක nimal123@gmail.com.</t>
         </is>
       </c>
-      <c r="E47" s="2" t="n"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>email id එක nimal123@gmail.කොම්.</t>
+        </is>
+      </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Inputs with Emojis</t>
+          <t>Inputs with Dates</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Contains emoji character embedded in Sinhala text</t>
+          <t>Contains date formats like "June 30", "15/07/2026"</t>
         </is>
       </c>
     </row>
@@ -2434,20 +2466,24 @@
           <t>ඔයාට සුබ දවසක් 😊, but ඒ message එක ignore කරන්න එපා.</t>
         </is>
       </c>
-      <c r="E48" s="2" t="n"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>ඔයාට සුබ දවසක් 😊, but ඒ message එක ignore කරන්න එපා.</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Inputs with Emojis</t>
+          <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Contains emoji character embedded in Sinhala text</t>
+          <t>Contains measurement units like "2 hours", "meters", "kilograms"</t>
         </is>
       </c>
     </row>
@@ -2474,22 +2510,22 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>ඔයාට සුබ දවසක් 😊, but ඒ message එක ignore කරන්න එපා.</t>
+          <t>මම හොඳ mood එකේ ඉන්නේ 😎, yet ඌයි update කරන්න එපා.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Inputs with Code-Switching</t>
+          <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Full code-switching between Sinhala and English: "then call me asap, otherwise text karanna"</t>
+          <t>Contains measurement units like "meters", "kilograms", "220V"</t>
         </is>
       </c>
     </row>
@@ -2516,22 +2552,22 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>මම හොඳ mood එකේ ඉන්නේ 😎, yet ඌයි update කරන්න එපා.</t>
+          <t>ඔයා එනවද? then call me asap, වෙනත්වසේ text කරන්න.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Inputs with Code-Switching</t>
+          <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Full code-switching with English phrase: "buddy, and this is urgent pls"</t>
+          <t>Uses slang/informal language</t>
         </is>
       </c>
     </row>
@@ -2558,12 +2594,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>ඔයා එනවද? then call me asap, වෙනත්වසේ text කරන්න.</t>
+          <t>මට පොඩ්ඩක් උදව් කරන්න, buddy, and this is urgent please.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">

</xml_diff>